<commit_message>
Add Kruskal-Wallis analysis and results documentation
- Introduced a new Python script for batch Kruskal-Wallis analysis (`kruskal_batch_analysis.py`) to evaluate mechanical accuracy across multiple factors.
- Added an Excel output file (`adjusted_position_kruskal_results.xlsx`) to store analysis results.
- Created a markdown file (`adjusted_position_kruskal_significance.md`) summarizing the significance findings from the analysis.
- Included new figures related to work envelope and mechanical accuracy in the `work_env` directory.
- Updated `requirements.txt` to include necessary libraries for statistical analysis.
- Documented statistical methods and results in a new Word document (`manuscript_section.docx`).
</commit_message>
<xml_diff>
--- a/figures/master_error.xlsx
+++ b/figures/master_error.xlsx
@@ -1,20 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adityakulkarni/Downloads/error_cal/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NavineticsAI\tools\m1-gtf\figures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1369635-2849-B043-B3A3-B8242F7FBDDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9BD3A34-4445-449B-AFD2-981112EA40F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="580" windowWidth="25600" windowHeight="16060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-46176" yWindow="1044" windowWidth="23232" windowHeight="18576" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="adjusted_position" sheetId="1" r:id="rId1"/>
     <sheet name="adapter" sheetId="2" r:id="rId2"/>
+    <sheet name="adapter_fig" sheetId="4" r:id="rId3"/>
+    <sheet name="comparison" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -37,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="31">
   <si>
     <t>target_id</t>
   </si>
@@ -96,22 +98,10 @@
     <t>L</t>
   </si>
   <si>
-    <t>MAH</t>
-  </si>
-  <si>
-    <t>CO</t>
-  </si>
-  <si>
-    <t>AK</t>
-  </si>
-  <si>
     <t>T2</t>
   </si>
   <si>
     <t>T3L</t>
-  </si>
-  <si>
-    <t>M</t>
   </si>
   <si>
     <t>T3R</t>
@@ -125,12 +115,30 @@
   <si>
     <t>T5</t>
   </si>
+  <si>
+    <t>method</t>
+  </si>
+  <si>
+    <t>adapter</t>
+  </si>
+  <si>
+    <t>adjusted</t>
+  </si>
+  <si>
+    <t>OP1</t>
+  </si>
+  <si>
+    <t>OP2</t>
+  </si>
+  <si>
+    <t>OP3</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -151,6 +159,12 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -165,7 +179,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -188,11 +202,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -204,6 +229,12 @@
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -221,10 +252,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -545,22 +572,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.83984375" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="8.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="4" width="4.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="4.5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.1640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.15625" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="4.47265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.3125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.47265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="4.47265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.83984375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.15625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.3125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="8" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="4.33203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="17" width="16.6640625" customWidth="1"/>
+    <col min="12" max="12" width="4.3125" bestFit="1" customWidth="1"/>
+    <col min="13" max="17" width="16.68359375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -613,7 +640,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="3" t="s">
         <v>17</v>
       </c>
@@ -644,8 +671,8 @@
       <c r="J2" s="3">
         <v>142.69999999999999</v>
       </c>
-      <c r="K2" s="3" t="s">
-        <v>19</v>
+      <c r="K2" s="1" t="s">
+        <v>28</v>
       </c>
       <c r="L2" s="3">
         <v>1</v>
@@ -668,7 +695,7 @@
         <v>1.3768951625060992</v>
       </c>
     </row>
-    <row r="3" spans="1:17" ht="16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="3" t="s">
         <v>17</v>
       </c>
@@ -699,8 +726,8 @@
       <c r="J3" s="3">
         <v>142.69999999999999</v>
       </c>
-      <c r="K3" s="3" t="s">
-        <v>20</v>
+      <c r="K3" s="1" t="s">
+        <v>29</v>
       </c>
       <c r="L3" s="3">
         <v>1</v>
@@ -723,7 +750,7 @@
         <v>1.1434249026830265</v>
       </c>
     </row>
-    <row r="4" spans="1:17" ht="16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="3" t="s">
         <v>17</v>
       </c>
@@ -754,8 +781,8 @@
       <c r="J4" s="3">
         <v>142.69999999999999</v>
       </c>
-      <c r="K4" s="3" t="s">
-        <v>21</v>
+      <c r="K4" s="1" t="s">
+        <v>30</v>
       </c>
       <c r="L4" s="3">
         <v>1</v>
@@ -778,9 +805,9 @@
         <v>1.3661568623994826</v>
       </c>
     </row>
-    <row r="5" spans="1:17" ht="16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B5" s="3">
         <v>140</v>
@@ -809,8 +836,8 @@
       <c r="J5" s="3">
         <v>70</v>
       </c>
-      <c r="K5" s="3" t="s">
-        <v>19</v>
+      <c r="K5" s="1" t="s">
+        <v>28</v>
       </c>
       <c r="L5" s="3">
         <v>1</v>
@@ -833,9 +860,9 @@
         <v>1.2673200069437869</v>
       </c>
     </row>
-    <row r="6" spans="1:17" ht="16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B6" s="3">
         <v>140</v>
@@ -864,8 +891,8 @@
       <c r="J6" s="3">
         <v>70</v>
       </c>
-      <c r="K6" s="3" t="s">
-        <v>20</v>
+      <c r="K6" s="1" t="s">
+        <v>29</v>
       </c>
       <c r="L6" s="3">
         <v>1</v>
@@ -888,9 +915,9 @@
         <v>1.4601369798755184</v>
       </c>
     </row>
-    <row r="7" spans="1:17" ht="16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B7" s="3">
         <v>140</v>
@@ -919,8 +946,8 @@
       <c r="J7" s="3">
         <v>70</v>
       </c>
-      <c r="K7" s="3" t="s">
-        <v>21</v>
+      <c r="K7" s="1" t="s">
+        <v>30</v>
       </c>
       <c r="L7" s="3">
         <v>1</v>
@@ -943,9 +970,9 @@
         <v>1.067988763985839</v>
       </c>
     </row>
-    <row r="8" spans="1:17" ht="16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="3" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B8" s="3">
         <v>100</v>
@@ -957,7 +984,7 @@
         <v>90</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="F8" s="3">
         <v>75</v>
@@ -974,8 +1001,8 @@
       <c r="J8" s="3">
         <v>97.3</v>
       </c>
-      <c r="K8" s="3" t="s">
-        <v>19</v>
+      <c r="K8" s="1" t="s">
+        <v>28</v>
       </c>
       <c r="L8" s="3">
         <v>1</v>
@@ -998,9 +1025,9 @@
         <v>0.63386278665240725</v>
       </c>
     </row>
-    <row r="9" spans="1:17" ht="16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="3" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B9" s="3">
         <v>100</v>
@@ -1012,7 +1039,7 @@
         <v>90</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="F9" s="3">
         <v>75</v>
@@ -1029,8 +1056,8 @@
       <c r="J9" s="3">
         <v>97.3</v>
       </c>
-      <c r="K9" s="3" t="s">
-        <v>20</v>
+      <c r="K9" s="1" t="s">
+        <v>29</v>
       </c>
       <c r="L9" s="3">
         <v>1</v>
@@ -1053,9 +1080,9 @@
         <v>0.57102639446027337</v>
       </c>
     </row>
-    <row r="10" spans="1:17" ht="16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="3" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B10" s="3">
         <v>100</v>
@@ -1067,7 +1094,7 @@
         <v>90</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="F10" s="3">
         <v>75</v>
@@ -1084,8 +1111,8 @@
       <c r="J10" s="3">
         <v>97.3</v>
       </c>
-      <c r="K10" s="3" t="s">
-        <v>21</v>
+      <c r="K10" s="1" t="s">
+        <v>30</v>
       </c>
       <c r="L10" s="3">
         <v>1</v>
@@ -1108,9 +1135,9 @@
         <v>0.89568586874699263</v>
       </c>
     </row>
-    <row r="11" spans="1:17" ht="16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="3" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B11" s="3">
         <v>100</v>
@@ -1122,7 +1149,7 @@
         <v>90</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F11" s="3">
         <v>75</v>
@@ -1139,8 +1166,8 @@
       <c r="J11" s="3">
         <v>97.3</v>
       </c>
-      <c r="K11" s="3" t="s">
-        <v>19</v>
+      <c r="K11" s="1" t="s">
+        <v>28</v>
       </c>
       <c r="L11" s="3">
         <v>1</v>
@@ -1163,9 +1190,9 @@
         <v>1.3046620626496495</v>
       </c>
     </row>
-    <row r="12" spans="1:17" ht="16" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="3" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B12" s="3">
         <v>100</v>
@@ -1177,7 +1204,7 @@
         <v>90</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F12" s="3">
         <v>75</v>
@@ -1194,8 +1221,8 @@
       <c r="J12" s="3">
         <v>97.3</v>
       </c>
-      <c r="K12" s="3" t="s">
-        <v>20</v>
+      <c r="K12" s="1" t="s">
+        <v>29</v>
       </c>
       <c r="L12" s="3">
         <v>1</v>
@@ -1218,9 +1245,9 @@
         <v>0.75537928655044728</v>
       </c>
     </row>
-    <row r="13" spans="1:17" ht="16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="3" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B13" s="3">
         <v>100</v>
@@ -1232,7 +1259,7 @@
         <v>90</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F13" s="3">
         <v>75</v>
@@ -1249,8 +1276,8 @@
       <c r="J13" s="3">
         <v>97.3</v>
       </c>
-      <c r="K13" s="3" t="s">
-        <v>21</v>
+      <c r="K13" s="1" t="s">
+        <v>30</v>
       </c>
       <c r="L13" s="3">
         <v>1</v>
@@ -1273,9 +1300,9 @@
         <v>1.1636004535436917</v>
       </c>
     </row>
-    <row r="14" spans="1:17" ht="16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B14" s="3">
         <v>60</v>
@@ -1287,7 +1314,7 @@
         <v>80</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F14" s="3">
         <v>75</v>
@@ -1304,8 +1331,8 @@
       <c r="J14" s="3">
         <v>134.6</v>
       </c>
-      <c r="K14" s="3" t="s">
-        <v>19</v>
+      <c r="K14" s="1" t="s">
+        <v>28</v>
       </c>
       <c r="L14" s="3">
         <v>1</v>
@@ -1328,9 +1355,9 @@
         <v>2.1102052595344496</v>
       </c>
     </row>
-    <row r="15" spans="1:17" ht="16" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B15" s="3">
         <v>60</v>
@@ -1342,7 +1369,7 @@
         <v>80</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F15" s="3">
         <v>75</v>
@@ -1359,8 +1386,8 @@
       <c r="J15" s="3">
         <v>134.6</v>
       </c>
-      <c r="K15" s="3" t="s">
-        <v>20</v>
+      <c r="K15" s="1" t="s">
+        <v>29</v>
       </c>
       <c r="L15" s="3">
         <v>1</v>
@@ -1383,9 +1410,9 @@
         <v>1.2846813489644608</v>
       </c>
     </row>
-    <row r="16" spans="1:17" ht="16" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B16" s="3">
         <v>60</v>
@@ -1397,7 +1424,7 @@
         <v>80</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F16" s="3">
         <v>75</v>
@@ -1414,8 +1441,8 @@
       <c r="J16" s="3">
         <v>134.6</v>
       </c>
-      <c r="K16" s="3" t="s">
-        <v>21</v>
+      <c r="K16" s="1" t="s">
+        <v>30</v>
       </c>
       <c r="L16" s="3">
         <v>1</v>
@@ -1438,9 +1465,9 @@
         <v>1.1894796726578265</v>
       </c>
     </row>
-    <row r="17" spans="1:17" ht="16" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="3" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B17" s="3">
         <v>60</v>
@@ -1452,7 +1479,7 @@
         <v>100</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F17" s="3">
         <v>75</v>
@@ -1469,8 +1496,8 @@
       <c r="J17" s="3">
         <v>70</v>
       </c>
-      <c r="K17" s="3" t="s">
-        <v>19</v>
+      <c r="K17" s="1" t="s">
+        <v>28</v>
       </c>
       <c r="L17" s="3">
         <v>1</v>
@@ -1493,9 +1520,9 @@
         <v>0.62722727027758562</v>
       </c>
     </row>
-    <row r="18" spans="1:17" ht="16" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:17" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="3" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B18" s="3">
         <v>60</v>
@@ -1507,7 +1534,7 @@
         <v>100</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F18" s="3">
         <v>75</v>
@@ -1524,8 +1551,8 @@
       <c r="J18" s="3">
         <v>70</v>
       </c>
-      <c r="K18" s="3" t="s">
-        <v>20</v>
+      <c r="K18" s="1" t="s">
+        <v>29</v>
       </c>
       <c r="L18" s="3">
         <v>1</v>
@@ -1548,9 +1575,9 @@
         <v>2.3503569043603498</v>
       </c>
     </row>
-    <row r="19" spans="1:17" ht="16" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:17" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="3" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B19" s="3">
         <v>60</v>
@@ -1562,7 +1589,7 @@
         <v>100</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F19" s="3">
         <v>75</v>
@@ -1579,8 +1606,8 @@
       <c r="J19" s="3">
         <v>70</v>
       </c>
-      <c r="K19" s="3" t="s">
-        <v>21</v>
+      <c r="K19" s="1" t="s">
+        <v>30</v>
       </c>
       <c r="L19" s="3">
         <v>1</v>
@@ -1615,15 +1642,16 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB6E8834-3208-48DC-9A4D-1D8F020BCC1B}">
   <dimension ref="A1:L19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.83984375" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1661,7 +1689,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="1" t="s">
         <v>17</v>
       </c>
@@ -1679,18 +1707,17 @@
       </c>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
-      <c r="H2" s="1">
-        <v>1</v>
+      <c r="H2" s="1" t="s">
+        <v>28</v>
       </c>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
       <c r="L2" s="1">
-        <f t="shared" ref="L2:L19" si="0">SQRT(SUMSQ(I2,J2,K2))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="1" t="s">
         <v>17</v>
       </c>
@@ -1708,18 +1735,17 @@
       </c>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
-      <c r="H3" s="1">
-        <v>2</v>
+      <c r="H3" s="1" t="s">
+        <v>29</v>
       </c>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1">
-        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="1" t="s">
         <v>17</v>
       </c>
@@ -1737,20 +1763,19 @@
       </c>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
-      <c r="H4" s="1">
-        <v>3</v>
+      <c r="H4" s="1" t="s">
+        <v>30</v>
       </c>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
       <c r="L4" s="1">
-        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="1" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B5" s="1">
         <v>140</v>
@@ -1765,31 +1790,30 @@
         <v>18</v>
       </c>
       <c r="F5" s="1">
-        <v>55</v>
+        <v>90</v>
       </c>
       <c r="G5" s="1">
-        <v>105</v>
-      </c>
-      <c r="H5" s="1">
-        <v>1</v>
+        <v>100</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>28</v>
       </c>
       <c r="I5" s="1">
-        <v>0.9</v>
+        <v>0.87</v>
       </c>
       <c r="J5" s="1">
-        <v>0.5</v>
+        <v>1.9</v>
       </c>
       <c r="K5" s="1">
-        <v>0.9</v>
+        <v>1.3</v>
       </c>
       <c r="L5" s="1">
-        <f t="shared" si="0"/>
-        <v>1.3674794331177345</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+        <v>2.4610770000144249</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="1" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B6" s="1">
         <v>140</v>
@@ -1804,31 +1828,30 @@
         <v>18</v>
       </c>
       <c r="F6" s="1">
-        <v>55</v>
+        <v>90</v>
       </c>
       <c r="G6" s="1">
-        <v>105</v>
-      </c>
-      <c r="H6" s="1">
-        <v>2</v>
+        <v>100</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>29</v>
       </c>
       <c r="I6" s="1">
+        <v>1.19</v>
+      </c>
+      <c r="J6" s="1">
         <v>0.8</v>
       </c>
-      <c r="J6" s="1">
-        <v>0.5</v>
-      </c>
       <c r="K6" s="1">
-        <v>0.1</v>
+        <v>0.47</v>
       </c>
       <c r="L6" s="1">
-        <f t="shared" si="0"/>
-        <v>0.94868329805051388</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+        <v>1.5089731607951149</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="1" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B7" s="1">
         <v>140</v>
@@ -1843,31 +1866,30 @@
         <v>18</v>
       </c>
       <c r="F7" s="1">
-        <v>55</v>
+        <v>90</v>
       </c>
       <c r="G7" s="1">
-        <v>105</v>
-      </c>
-      <c r="H7" s="1">
-        <v>3</v>
+        <v>100</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>30</v>
       </c>
       <c r="I7" s="1">
-        <v>0.9</v>
+        <v>0.92</v>
       </c>
       <c r="J7" s="1">
-        <v>0.5</v>
+        <v>0.98</v>
       </c>
       <c r="K7" s="1">
-        <v>0.3</v>
+        <v>1.23</v>
       </c>
       <c r="L7" s="1">
-        <f t="shared" si="0"/>
-        <v>1.0723805294763609</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+        <v>1.8220043907740728</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="1" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B8" s="1">
         <v>100</v>
@@ -1879,24 +1901,33 @@
         <v>90</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1">
-        <v>1</v>
-      </c>
-      <c r="I8" s="1"/>
-      <c r="J8" s="1"/>
-      <c r="K8" s="1"/>
+        <v>18</v>
+      </c>
+      <c r="F8" s="1">
+        <v>75</v>
+      </c>
+      <c r="G8" s="1">
+        <v>105</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I8" s="1">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="J8" s="1">
+        <v>1.38</v>
+      </c>
+      <c r="K8" s="1">
+        <v>0.92</v>
+      </c>
       <c r="L8" s="1">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+        <v>1.7570429704477919</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="1" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B9" s="1">
         <v>100</v>
@@ -1908,24 +1939,33 @@
         <v>90</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="F9" s="1"/>
-      <c r="G9" s="1"/>
-      <c r="H9" s="1">
-        <v>2</v>
-      </c>
-      <c r="I9" s="1"/>
-      <c r="J9" s="1"/>
-      <c r="K9" s="1"/>
+        <v>18</v>
+      </c>
+      <c r="F9" s="1">
+        <v>75</v>
+      </c>
+      <c r="G9" s="1">
+        <v>105</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="I9" s="1">
+        <v>0</v>
+      </c>
+      <c r="J9" s="1">
+        <v>0.62</v>
+      </c>
+      <c r="K9" s="1">
+        <v>0.16</v>
+      </c>
       <c r="L9" s="1">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+        <v>0.6403124237432849</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="1" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B10" s="1">
         <v>100</v>
@@ -1937,24 +1977,33 @@
         <v>90</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="F10" s="1"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="1">
-        <v>3</v>
-      </c>
-      <c r="I10" s="1"/>
-      <c r="J10" s="1"/>
-      <c r="K10" s="1"/>
+        <v>18</v>
+      </c>
+      <c r="F10" s="1">
+        <v>75</v>
+      </c>
+      <c r="G10" s="1">
+        <v>105</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I10" s="1">
+        <v>0.78</v>
+      </c>
+      <c r="J10" s="1">
+        <v>0.89</v>
+      </c>
+      <c r="K10" s="1">
+        <v>1.1000000000000001</v>
+      </c>
       <c r="L10" s="1">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+        <v>1.6157041808449961</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="1" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B11" s="1">
         <v>100</v>
@@ -1966,34 +2015,33 @@
         <v>90</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F11" s="1">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="G11" s="1">
-        <v>60</v>
-      </c>
-      <c r="H11" s="1">
-        <v>1</v>
+        <v>75</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>28</v>
       </c>
       <c r="I11" s="1">
+        <v>0.98</v>
+      </c>
+      <c r="J11" s="1">
+        <v>1.05</v>
+      </c>
+      <c r="K11" s="1">
         <v>0.5</v>
       </c>
-      <c r="J11" s="1">
-        <v>0.2</v>
-      </c>
-      <c r="K11" s="1">
-        <v>0.9</v>
-      </c>
       <c r="L11" s="1">
-        <f t="shared" si="0"/>
-        <v>1.0488088481701516</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+        <v>1.5208221460775746</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="1" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B12" s="1">
         <v>100</v>
@@ -2005,34 +2053,33 @@
         <v>90</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F12" s="1">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="G12" s="1">
-        <v>60</v>
-      </c>
-      <c r="H12" s="1">
-        <v>2</v>
+        <v>75</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>29</v>
       </c>
       <c r="I12" s="1">
-        <v>1</v>
+        <v>0.47</v>
       </c>
       <c r="J12" s="1">
-        <v>0.1</v>
+        <v>0.41</v>
       </c>
       <c r="K12" s="1">
-        <v>0.3</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="L12" s="1">
-        <f t="shared" si="0"/>
-        <v>1.0488088481701516</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+        <v>0.68366658540548841</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="1" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B13" s="1">
         <v>100</v>
@@ -2044,34 +2091,33 @@
         <v>90</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F13" s="1">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="G13" s="1">
-        <v>60</v>
-      </c>
-      <c r="H13" s="1">
-        <v>3</v>
+        <v>75</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>30</v>
       </c>
       <c r="I13" s="1">
-        <v>0.8</v>
+        <v>0.98</v>
       </c>
       <c r="J13" s="1">
-        <v>0.1</v>
+        <v>0.87</v>
       </c>
       <c r="K13" s="1">
-        <v>0.1</v>
+        <v>1.08</v>
       </c>
       <c r="L13" s="1">
-        <f t="shared" si="0"/>
-        <v>0.81240384046359615</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+        <v>1.6981460479004744</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="1" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B14" s="1">
         <v>60</v>
@@ -2083,34 +2129,33 @@
         <v>80</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F14" s="1">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="G14" s="1">
-        <v>60</v>
-      </c>
-      <c r="H14" s="1">
-        <v>1</v>
+        <v>80</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>28</v>
       </c>
       <c r="I14" s="1">
-        <v>0.8</v>
+        <v>0.63</v>
       </c>
       <c r="J14" s="1">
-        <v>1.1000000000000001</v>
+        <v>1.45</v>
       </c>
       <c r="K14" s="1">
-        <v>0.1</v>
+        <v>0.48</v>
       </c>
       <c r="L14" s="1">
-        <f t="shared" si="0"/>
-        <v>1.3638181696985856</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+        <v>1.6522106403240477</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="1" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B15" s="1">
         <v>60</v>
@@ -2122,34 +2167,33 @@
         <v>80</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F15" s="1">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="G15" s="1">
-        <v>60</v>
-      </c>
-      <c r="H15" s="1">
-        <v>2</v>
+        <v>80</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>29</v>
       </c>
       <c r="I15" s="1">
-        <v>1.5</v>
+        <v>0.9</v>
       </c>
       <c r="J15" s="1">
-        <v>0.4</v>
+        <v>1.92</v>
       </c>
       <c r="K15" s="1">
-        <v>0.1</v>
+        <v>1.3</v>
       </c>
       <c r="L15" s="1">
-        <f t="shared" si="0"/>
-        <v>1.5556349186104046</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+        <v>2.487247474619283</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="1" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B16" s="1">
         <v>60</v>
@@ -2161,34 +2205,33 @@
         <v>80</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F16" s="1">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="G16" s="1">
-        <v>60</v>
-      </c>
-      <c r="H16" s="1">
-        <v>3</v>
+        <v>80</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>30</v>
       </c>
       <c r="I16" s="1">
-        <v>1.6</v>
+        <v>0.43</v>
       </c>
       <c r="J16" s="1">
-        <v>0.6</v>
+        <v>0.94</v>
       </c>
       <c r="K16" s="1">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="L16" s="1">
-        <f t="shared" si="0"/>
-        <v>1.7204650534085255</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+        <v>1.0385085459446157</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="1" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B17" s="1">
         <v>60</v>
@@ -2200,34 +2243,33 @@
         <v>100</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F17" s="1">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="G17" s="1">
-        <v>60</v>
-      </c>
-      <c r="H17" s="1">
-        <v>1</v>
+        <v>80</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>28</v>
       </c>
       <c r="I17" s="1">
-        <v>0.8</v>
+        <v>0.2</v>
       </c>
       <c r="J17" s="1">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="K17" s="1">
-        <v>0.2</v>
+        <v>0.68</v>
       </c>
       <c r="L17" s="1">
-        <f t="shared" si="0"/>
-        <v>0.83066238629180755</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+        <v>0.73647810558087878</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="1" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B18" s="1">
         <v>60</v>
@@ -2239,34 +2281,33 @@
         <v>100</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F18" s="1">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="G18" s="1">
-        <v>60</v>
-      </c>
-      <c r="H18" s="1">
-        <v>2</v>
+        <v>80</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>29</v>
       </c>
       <c r="I18" s="1">
-        <v>1.5</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="J18" s="1">
-        <v>0.1</v>
+        <v>1.74</v>
       </c>
       <c r="K18" s="1">
-        <v>0.3</v>
+        <v>1.18</v>
       </c>
       <c r="L18" s="1">
-        <f t="shared" si="0"/>
-        <v>1.532970971675589</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+        <v>2.173131381210073</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="1" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B19" s="1">
         <v>60</v>
@@ -2278,32 +2319,32 @@
         <v>100</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F19" s="1">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="G19" s="1">
-        <v>60</v>
-      </c>
-      <c r="H19" s="1">
-        <v>3</v>
+        <v>80</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>30</v>
       </c>
       <c r="I19" s="1">
-        <v>1.1000000000000001</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="J19" s="1">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="K19" s="1">
-        <v>0.1</v>
+        <v>0.34</v>
       </c>
       <c r="L19" s="1">
-        <f t="shared" si="0"/>
-        <v>1.2569805089976536</v>
+        <v>1.1131936040060597</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="L2:L19">
     <cfRule type="colorScale" priority="1">
       <colorScale>
@@ -2324,4 +2365,1570 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE99BABF-A6A7-4E2C-ACE3-2941007B8434}">
+  <dimension ref="A1:L16"/>
+  <sheetFormatPr defaultColWidth="8.83984375" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="1">
+        <v>140</v>
+      </c>
+      <c r="C2" s="1">
+        <v>70</v>
+      </c>
+      <c r="D2" s="1">
+        <v>70</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" s="1">
+        <v>90</v>
+      </c>
+      <c r="G2" s="1">
+        <v>100</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I2" s="1">
+        <v>0.87</v>
+      </c>
+      <c r="J2" s="1">
+        <v>1.9</v>
+      </c>
+      <c r="K2" s="1">
+        <v>1.3</v>
+      </c>
+      <c r="L2" s="1">
+        <v>2.4610770000144249</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="1">
+        <v>140</v>
+      </c>
+      <c r="C3" s="1">
+        <v>70</v>
+      </c>
+      <c r="D3" s="1">
+        <v>70</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="1">
+        <v>90</v>
+      </c>
+      <c r="G3" s="1">
+        <v>100</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="I3" s="1">
+        <v>1.19</v>
+      </c>
+      <c r="J3" s="1">
+        <v>0.8</v>
+      </c>
+      <c r="K3" s="1">
+        <v>0.47</v>
+      </c>
+      <c r="L3" s="1">
+        <v>1.5089731607951149</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="1">
+        <v>140</v>
+      </c>
+      <c r="C4" s="1">
+        <v>70</v>
+      </c>
+      <c r="D4" s="1">
+        <v>70</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" s="1">
+        <v>90</v>
+      </c>
+      <c r="G4" s="1">
+        <v>100</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I4" s="1">
+        <v>0.92</v>
+      </c>
+      <c r="J4" s="1">
+        <v>0.98</v>
+      </c>
+      <c r="K4" s="1">
+        <v>1.23</v>
+      </c>
+      <c r="L4" s="1">
+        <v>1.8220043907740728</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="1">
+        <v>100</v>
+      </c>
+      <c r="C5" s="1">
+        <v>100</v>
+      </c>
+      <c r="D5" s="1">
+        <v>90</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" s="1">
+        <v>75</v>
+      </c>
+      <c r="G5" s="1">
+        <v>105</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I5" s="1">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="J5" s="1">
+        <v>1.38</v>
+      </c>
+      <c r="K5" s="1">
+        <v>0.92</v>
+      </c>
+      <c r="L5" s="1">
+        <v>1.7570429704477919</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="1">
+        <v>100</v>
+      </c>
+      <c r="C6" s="1">
+        <v>100</v>
+      </c>
+      <c r="D6" s="1">
+        <v>90</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" s="1">
+        <v>75</v>
+      </c>
+      <c r="G6" s="1">
+        <v>105</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="I6" s="1">
+        <v>0</v>
+      </c>
+      <c r="J6" s="1">
+        <v>0.62</v>
+      </c>
+      <c r="K6" s="1">
+        <v>0.16</v>
+      </c>
+      <c r="L6" s="1">
+        <v>0.6403124237432849</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A7" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="1">
+        <v>100</v>
+      </c>
+      <c r="C7" s="1">
+        <v>100</v>
+      </c>
+      <c r="D7" s="1">
+        <v>90</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F7" s="1">
+        <v>75</v>
+      </c>
+      <c r="G7" s="1">
+        <v>105</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I7" s="1">
+        <v>0.78</v>
+      </c>
+      <c r="J7" s="1">
+        <v>0.89</v>
+      </c>
+      <c r="K7" s="1">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="L7" s="1">
+        <v>1.6157041808449961</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A8" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="1">
+        <v>100</v>
+      </c>
+      <c r="C8" s="1">
+        <v>100</v>
+      </c>
+      <c r="D8" s="1">
+        <v>90</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F8" s="1">
+        <v>75</v>
+      </c>
+      <c r="G8" s="1">
+        <v>75</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I8" s="1">
+        <v>0.98</v>
+      </c>
+      <c r="J8" s="1">
+        <v>1.05</v>
+      </c>
+      <c r="K8" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="L8" s="1">
+        <v>1.5208221460775746</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9" s="1">
+        <v>100</v>
+      </c>
+      <c r="C9" s="1">
+        <v>100</v>
+      </c>
+      <c r="D9" s="1">
+        <v>90</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F9" s="1">
+        <v>75</v>
+      </c>
+      <c r="G9" s="1">
+        <v>75</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="I9" s="1">
+        <v>0.47</v>
+      </c>
+      <c r="J9" s="1">
+        <v>0.41</v>
+      </c>
+      <c r="K9" s="1">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="L9" s="1">
+        <v>0.68366658540548841</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A10" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="1">
+        <v>100</v>
+      </c>
+      <c r="C10" s="1">
+        <v>100</v>
+      </c>
+      <c r="D10" s="1">
+        <v>90</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F10" s="1">
+        <v>75</v>
+      </c>
+      <c r="G10" s="1">
+        <v>75</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I10" s="1">
+        <v>0.98</v>
+      </c>
+      <c r="J10" s="1">
+        <v>0.87</v>
+      </c>
+      <c r="K10" s="1">
+        <v>1.08</v>
+      </c>
+      <c r="L10" s="1">
+        <v>1.6981460479004744</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A11" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="1">
+        <v>60</v>
+      </c>
+      <c r="C11" s="1">
+        <v>140</v>
+      </c>
+      <c r="D11" s="1">
+        <v>80</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F11" s="1">
+        <v>75</v>
+      </c>
+      <c r="G11" s="1">
+        <v>80</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I11" s="1">
+        <v>0.63</v>
+      </c>
+      <c r="J11" s="1">
+        <v>1.45</v>
+      </c>
+      <c r="K11" s="1">
+        <v>0.48</v>
+      </c>
+      <c r="L11" s="1">
+        <v>1.6522106403240477</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A12" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="1">
+        <v>60</v>
+      </c>
+      <c r="C12" s="1">
+        <v>140</v>
+      </c>
+      <c r="D12" s="1">
+        <v>80</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F12" s="1">
+        <v>75</v>
+      </c>
+      <c r="G12" s="1">
+        <v>80</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="I12" s="1">
+        <v>0.9</v>
+      </c>
+      <c r="J12" s="1">
+        <v>1.92</v>
+      </c>
+      <c r="K12" s="1">
+        <v>1.3</v>
+      </c>
+      <c r="L12" s="1">
+        <v>2.487247474619283</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A13" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" s="1">
+        <v>60</v>
+      </c>
+      <c r="C13" s="1">
+        <v>140</v>
+      </c>
+      <c r="D13" s="1">
+        <v>80</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F13" s="1">
+        <v>75</v>
+      </c>
+      <c r="G13" s="1">
+        <v>80</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I13" s="1">
+        <v>0.43</v>
+      </c>
+      <c r="J13" s="1">
+        <v>0.94</v>
+      </c>
+      <c r="K13" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="L13" s="1">
+        <v>1.0385085459446157</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A14" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="1">
+        <v>60</v>
+      </c>
+      <c r="C14" s="1">
+        <v>70</v>
+      </c>
+      <c r="D14" s="1">
+        <v>100</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F14" s="1">
+        <v>75</v>
+      </c>
+      <c r="G14" s="1">
+        <v>80</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I14" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="J14" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="K14" s="1">
+        <v>0.68</v>
+      </c>
+      <c r="L14" s="1">
+        <v>0.73647810558087878</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A15" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B15" s="1">
+        <v>60</v>
+      </c>
+      <c r="C15" s="1">
+        <v>70</v>
+      </c>
+      <c r="D15" s="1">
+        <v>100</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F15" s="1">
+        <v>75</v>
+      </c>
+      <c r="G15" s="1">
+        <v>80</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="I15" s="1">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="J15" s="1">
+        <v>1.74</v>
+      </c>
+      <c r="K15" s="1">
+        <v>1.18</v>
+      </c>
+      <c r="L15" s="1">
+        <v>2.173131381210073</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A16" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" s="1">
+        <v>60</v>
+      </c>
+      <c r="C16" s="1">
+        <v>70</v>
+      </c>
+      <c r="D16" s="1">
+        <v>100</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F16" s="1">
+        <v>75</v>
+      </c>
+      <c r="G16" s="1">
+        <v>80</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I16" s="1">
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="J16" s="1">
+        <v>0.9</v>
+      </c>
+      <c r="K16" s="1">
+        <v>0.34</v>
+      </c>
+      <c r="L16" s="1">
+        <v>1.1131936040060597</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="L2:L16">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88237414-97E6-45C4-975D-88BC378D59C7}">
+  <dimension ref="A1:I31"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <cols>
+    <col min="6" max="6" width="15.734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="1">
+        <v>140</v>
+      </c>
+      <c r="C2" s="1">
+        <v>70</v>
+      </c>
+      <c r="D2" s="1">
+        <v>70</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F2" s="1">
+        <v>2.4610770000144249</v>
+      </c>
+      <c r="G2">
+        <v>0.87</v>
+      </c>
+      <c r="H2">
+        <v>1.9</v>
+      </c>
+      <c r="I2">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="1">
+        <v>140</v>
+      </c>
+      <c r="C3" s="1">
+        <v>70</v>
+      </c>
+      <c r="D3" s="1">
+        <v>70</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F3" s="1">
+        <v>1.5089731607951149</v>
+      </c>
+      <c r="G3">
+        <v>1.19</v>
+      </c>
+      <c r="H3">
+        <v>0.8</v>
+      </c>
+      <c r="I3">
+        <v>0.47</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="1">
+        <v>140</v>
+      </c>
+      <c r="C4" s="1">
+        <v>70</v>
+      </c>
+      <c r="D4" s="1">
+        <v>70</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" s="1">
+        <v>1.8220043907740728</v>
+      </c>
+      <c r="G4">
+        <v>0.92</v>
+      </c>
+      <c r="H4">
+        <v>0.98</v>
+      </c>
+      <c r="I4">
+        <v>1.23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="1">
+        <v>100</v>
+      </c>
+      <c r="C5" s="1">
+        <v>100</v>
+      </c>
+      <c r="D5" s="1">
+        <v>90</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" s="1">
+        <v>1.7570429704477919</v>
+      </c>
+      <c r="G5">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="H5">
+        <v>1.38</v>
+      </c>
+      <c r="I5">
+        <v>0.92</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="1">
+        <v>100</v>
+      </c>
+      <c r="C6" s="1">
+        <v>100</v>
+      </c>
+      <c r="D6" s="1">
+        <v>90</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F6" s="1">
+        <v>0.6403124237432849</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>0.62</v>
+      </c>
+      <c r="I6">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A7" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="1">
+        <v>100</v>
+      </c>
+      <c r="C7" s="1">
+        <v>100</v>
+      </c>
+      <c r="D7" s="1">
+        <v>90</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F7" s="1">
+        <v>1.6157041808449961</v>
+      </c>
+      <c r="G7">
+        <v>0.78</v>
+      </c>
+      <c r="H7">
+        <v>0.89</v>
+      </c>
+      <c r="I7">
+        <v>1.1000000000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A8" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="1">
+        <v>100</v>
+      </c>
+      <c r="C8" s="1">
+        <v>100</v>
+      </c>
+      <c r="D8" s="1">
+        <v>90</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F8" s="1">
+        <v>1.5208221460775746</v>
+      </c>
+      <c r="G8">
+        <v>0.98</v>
+      </c>
+      <c r="H8">
+        <v>1.05</v>
+      </c>
+      <c r="I8">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9" s="1">
+        <v>100</v>
+      </c>
+      <c r="C9" s="1">
+        <v>100</v>
+      </c>
+      <c r="D9" s="1">
+        <v>90</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F9" s="1">
+        <v>0.68366658540548841</v>
+      </c>
+      <c r="G9">
+        <v>0.47</v>
+      </c>
+      <c r="H9">
+        <v>0.41</v>
+      </c>
+      <c r="I9">
+        <v>0.28000000000000003</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A10" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="1">
+        <v>100</v>
+      </c>
+      <c r="C10" s="1">
+        <v>100</v>
+      </c>
+      <c r="D10" s="1">
+        <v>90</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F10" s="1">
+        <v>1.6981460479004744</v>
+      </c>
+      <c r="G10">
+        <v>0.98</v>
+      </c>
+      <c r="H10">
+        <v>0.87</v>
+      </c>
+      <c r="I10">
+        <v>1.08</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A11" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="1">
+        <v>60</v>
+      </c>
+      <c r="C11" s="1">
+        <v>140</v>
+      </c>
+      <c r="D11" s="1">
+        <v>80</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F11" s="1">
+        <v>1.6522106403240477</v>
+      </c>
+      <c r="G11">
+        <v>0.63</v>
+      </c>
+      <c r="H11">
+        <v>1.45</v>
+      </c>
+      <c r="I11">
+        <v>0.48</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A12" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="1">
+        <v>60</v>
+      </c>
+      <c r="C12" s="1">
+        <v>140</v>
+      </c>
+      <c r="D12" s="1">
+        <v>80</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F12" s="1">
+        <v>2.487247474619283</v>
+      </c>
+      <c r="G12">
+        <v>0.9</v>
+      </c>
+      <c r="H12">
+        <v>1.92</v>
+      </c>
+      <c r="I12">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A13" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" s="1">
+        <v>60</v>
+      </c>
+      <c r="C13" s="1">
+        <v>140</v>
+      </c>
+      <c r="D13" s="1">
+        <v>80</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F13" s="1">
+        <v>1.0385085459446157</v>
+      </c>
+      <c r="G13">
+        <v>0.43</v>
+      </c>
+      <c r="H13">
+        <v>0.94</v>
+      </c>
+      <c r="I13">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A14" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="1">
+        <v>60</v>
+      </c>
+      <c r="C14" s="1">
+        <v>70</v>
+      </c>
+      <c r="D14" s="1">
+        <v>100</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F14" s="1">
+        <v>0.73647810558087878</v>
+      </c>
+      <c r="G14">
+        <v>0.2</v>
+      </c>
+      <c r="H14">
+        <v>0.2</v>
+      </c>
+      <c r="I14">
+        <v>0.68</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A15" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B15" s="1">
+        <v>60</v>
+      </c>
+      <c r="C15" s="1">
+        <v>70</v>
+      </c>
+      <c r="D15" s="1">
+        <v>100</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F15" s="1">
+        <v>2.173131381210073</v>
+      </c>
+      <c r="G15">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="H15">
+        <v>1.74</v>
+      </c>
+      <c r="I15">
+        <v>1.18</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A16" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" s="1">
+        <v>60</v>
+      </c>
+      <c r="C16" s="1">
+        <v>70</v>
+      </c>
+      <c r="D16" s="1">
+        <v>100</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F16" s="1">
+        <v>1.1131936040060597</v>
+      </c>
+      <c r="G16">
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="H16">
+        <v>0.9</v>
+      </c>
+      <c r="I16">
+        <v>0.34</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A17" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="1">
+        <v>140</v>
+      </c>
+      <c r="C17" s="1">
+        <v>70</v>
+      </c>
+      <c r="D17" s="1">
+        <v>70</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F17">
+        <v>1.2673200069437869</v>
+      </c>
+      <c r="G17">
+        <v>0.2</v>
+      </c>
+      <c r="H17">
+        <v>1.25</v>
+      </c>
+      <c r="I17">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18" s="1">
+        <v>140</v>
+      </c>
+      <c r="C18" s="1">
+        <v>70</v>
+      </c>
+      <c r="D18" s="1">
+        <v>70</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F18">
+        <v>1.4601369798755184</v>
+      </c>
+      <c r="G18">
+        <v>0</v>
+      </c>
+      <c r="H18">
+        <v>1.46</v>
+      </c>
+      <c r="I18">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A19" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B19" s="1">
+        <v>140</v>
+      </c>
+      <c r="C19" s="1">
+        <v>70</v>
+      </c>
+      <c r="D19" s="1">
+        <v>70</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F19">
+        <v>1.067988763985839</v>
+      </c>
+      <c r="G19">
+        <v>0.46</v>
+      </c>
+      <c r="H19">
+        <v>0.37</v>
+      </c>
+      <c r="I19">
+        <v>0.89</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A20" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B20" s="1">
+        <v>100</v>
+      </c>
+      <c r="C20" s="1">
+        <v>100</v>
+      </c>
+      <c r="D20" s="1">
+        <v>90</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F20">
+        <v>0.63386278665240725</v>
+      </c>
+      <c r="G20">
+        <v>0.05</v>
+      </c>
+      <c r="H20">
+        <v>0.5</v>
+      </c>
+      <c r="I20">
+        <v>0.38637033051562736</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A21" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="1">
+        <v>100</v>
+      </c>
+      <c r="C21" s="1">
+        <v>100</v>
+      </c>
+      <c r="D21" s="1">
+        <v>90</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F21">
+        <v>0.57102639446027337</v>
+      </c>
+      <c r="G21">
+        <v>0.3</v>
+      </c>
+      <c r="H21">
+        <v>0.39</v>
+      </c>
+      <c r="I21">
+        <v>0.2897777478867205</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A22" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22" s="1">
+        <v>100</v>
+      </c>
+      <c r="C22" s="1">
+        <v>100</v>
+      </c>
+      <c r="D22" s="1">
+        <v>90</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F22">
+        <v>0.89568586874699263</v>
+      </c>
+      <c r="G22">
+        <v>0.59</v>
+      </c>
+      <c r="H22">
+        <v>0.47</v>
+      </c>
+      <c r="I22">
+        <v>0.48296291314453416</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A23" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B23" s="1">
+        <v>100</v>
+      </c>
+      <c r="C23" s="1">
+        <v>100</v>
+      </c>
+      <c r="D23" s="1">
+        <v>90</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F23">
+        <v>1.3046620626496495</v>
+      </c>
+      <c r="G23">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="H23">
+        <v>0.13</v>
+      </c>
+      <c r="I23">
+        <v>1.2653628324386796</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A24" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" s="1">
+        <v>100</v>
+      </c>
+      <c r="C24" s="1">
+        <v>100</v>
+      </c>
+      <c r="D24" s="1">
+        <v>90</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F24">
+        <v>0.75537928655044728</v>
+      </c>
+      <c r="G24">
+        <v>0.42</v>
+      </c>
+      <c r="H24">
+        <v>0</v>
+      </c>
+      <c r="I24">
+        <v>0.62785178708789446</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A25" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B25" s="1">
+        <v>100</v>
+      </c>
+      <c r="C25" s="1">
+        <v>100</v>
+      </c>
+      <c r="D25" s="1">
+        <v>90</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F25">
+        <v>1.1636004535436917</v>
+      </c>
+      <c r="G25">
+        <v>0.49</v>
+      </c>
+      <c r="H25">
+        <v>0.16</v>
+      </c>
+      <c r="I25">
+        <v>1.0431998923921939</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A26" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B26" s="1">
+        <v>60</v>
+      </c>
+      <c r="C26" s="1">
+        <v>140</v>
+      </c>
+      <c r="D26" s="1">
+        <v>80</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F26">
+        <v>2.1102052595344496</v>
+      </c>
+      <c r="G26">
+        <v>0.72</v>
+      </c>
+      <c r="H26">
+        <v>0.9</v>
+      </c>
+      <c r="I26">
+        <v>1.7676442621089952</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A27" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B27" s="1">
+        <v>60</v>
+      </c>
+      <c r="C27" s="1">
+        <v>140</v>
+      </c>
+      <c r="D27" s="1">
+        <v>80</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F27">
+        <v>1.2846813489644608</v>
+      </c>
+      <c r="G27">
+        <v>0</v>
+      </c>
+      <c r="H27">
+        <v>0</v>
+      </c>
+      <c r="I27">
+        <v>1.2846813489644608</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A28" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B28" s="1">
+        <v>60</v>
+      </c>
+      <c r="C28" s="1">
+        <v>140</v>
+      </c>
+      <c r="D28" s="1">
+        <v>80</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F28">
+        <v>1.1894796726578265</v>
+      </c>
+      <c r="G28">
+        <v>0.15</v>
+      </c>
+      <c r="H28">
+        <v>0.37</v>
+      </c>
+      <c r="I28">
+        <v>1.1204739584953192</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A29" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B29" s="1">
+        <v>60</v>
+      </c>
+      <c r="C29" s="1">
+        <v>70</v>
+      </c>
+      <c r="D29" s="1">
+        <v>100</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F29">
+        <v>0.62722727027758562</v>
+      </c>
+      <c r="G29">
+        <v>0</v>
+      </c>
+      <c r="H29">
+        <v>0.47</v>
+      </c>
+      <c r="I29">
+        <v>0.41534810530429939</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A30" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B30" s="1">
+        <v>60</v>
+      </c>
+      <c r="C30" s="1">
+        <v>70</v>
+      </c>
+      <c r="D30" s="1">
+        <v>100</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F30">
+        <v>2.3503569043603498</v>
+      </c>
+      <c r="G30">
+        <v>0.37</v>
+      </c>
+      <c r="H30">
+        <v>1.65</v>
+      </c>
+      <c r="I30">
+        <v>1.6324146464285254</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A31" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B31" s="1">
+        <v>60</v>
+      </c>
+      <c r="C31" s="1">
+        <v>70</v>
+      </c>
+      <c r="D31" s="1">
+        <v>100</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F31">
+        <v>0.59856211353723876</v>
+      </c>
+      <c r="G31">
+        <v>0</v>
+      </c>
+      <c r="H31">
+        <v>0.34</v>
+      </c>
+      <c r="I31">
+        <v>0.49262217140742487</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="F2:F16">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>